<commit_message>
Refactor Statuts Contractuels page
</commit_message>
<xml_diff>
--- a/public/data/contractuels.xlsx
+++ b/public/data/contractuels.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pcazenp5\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45497558-F7C5-4661-A2BA-2F523C460164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF295826-E277-482E-A1AB-DD1D8E217CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17235" yWindow="2805" windowWidth="21600" windowHeight="11235" xr2:uid="{0F3DF298-D4C5-439C-AF3F-C52F546A0520}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F3DF298-D4C5-439C-AF3F-C52F546A0520}"/>
   </bookViews>
   <sheets>
     <sheet name="contractuels" sheetId="2" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">contractuels!$A$1:$BZ$127</definedName>
     <definedName name="CODESTAT">#REF!</definedName>
@@ -6407,35 +6404,35 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="25" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="25" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -6457,51 +6454,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Corps"/>
-      <sheetName val="Grades"/>
-      <sheetName val="Statuts vacataires d'enseignem"/>
-      <sheetName val="Statuts vacataires"/>
-      <sheetName val="Statuts hébergés"/>
-      <sheetName val="Stat-emploi-pos. sans poste"/>
-      <sheetName val="Triplets"/>
-      <sheetName val="Positions"/>
-      <sheetName val="Modalités sc"/>
-      <sheetName val="Congés-absences"/>
-      <sheetName val="Emplois"/>
-      <sheetName val="Catégories d'emploi (plafond)"/>
-      <sheetName val="UO ED"/>
-      <sheetName val="Etablissements"/>
-      <sheetName val="Actes-visas-article"/>
-      <sheetName val="Diplômes"/>
-      <sheetName val="Mise à jour des référentiels"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6807,122 +6759,124 @@
   <dimension ref="A1:BZ128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="5.7109375" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.85546875" style="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="149.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="74.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="132.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="255.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="53.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="29.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="82.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="31.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.5703125" style="3" customWidth="1"/>
-    <col min="19" max="19" width="28.5703125" style="4" customWidth="1"/>
-    <col min="20" max="20" width="36.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="28.5703125" style="5" customWidth="1"/>
-    <col min="22" max="22" width="28.5703125" style="3" customWidth="1"/>
-    <col min="23" max="25" width="28.5703125" style="4" customWidth="1"/>
-    <col min="26" max="26" width="28.5703125" style="3" customWidth="1"/>
-    <col min="27" max="27" width="28.5703125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="33.42578125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="47.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="53.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="42.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="50.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="36.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="28.5703125" style="4" customWidth="1"/>
+    <col min="26" max="26" width="37.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="38.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="57.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="30" max="16384" width="5.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="206" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="209" t="s">
+    <row r="1" spans="1:29" s="204" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="207" t="s">
         <v>1015</v>
       </c>
-      <c r="B1" s="210" t="s">
+      <c r="B1" s="208" t="s">
         <v>1014</v>
       </c>
-      <c r="C1" s="209" t="s">
+      <c r="C1" s="207" t="s">
         <v>1013</v>
       </c>
-      <c r="D1" s="209" t="s">
+      <c r="D1" s="207" t="s">
         <v>1012</v>
       </c>
-      <c r="E1" s="209" t="s">
+      <c r="E1" s="207" t="s">
         <v>1011</v>
       </c>
-      <c r="F1" s="209" t="s">
+      <c r="F1" s="207" t="s">
         <v>1010</v>
       </c>
-      <c r="G1" s="209" t="s">
+      <c r="G1" s="207" t="s">
         <v>1009</v>
       </c>
-      <c r="H1" s="209" t="s">
+      <c r="H1" s="207" t="s">
         <v>1008</v>
       </c>
-      <c r="I1" s="209" t="s">
+      <c r="I1" s="207" t="s">
         <v>1007</v>
       </c>
-      <c r="J1" s="209" t="s">
+      <c r="J1" s="207" t="s">
         <v>1006</v>
       </c>
-      <c r="K1" s="209" t="s">
+      <c r="K1" s="207" t="s">
         <v>1005</v>
       </c>
-      <c r="L1" s="210" t="s">
+      <c r="L1" s="208" t="s">
         <v>1004</v>
       </c>
-      <c r="M1" s="210" t="s">
+      <c r="M1" s="208" t="s">
         <v>1003</v>
       </c>
-      <c r="N1" s="210" t="s">
+      <c r="N1" s="208" t="s">
         <v>1002</v>
       </c>
-      <c r="O1" s="210" t="s">
+      <c r="O1" s="208" t="s">
         <v>1001</v>
       </c>
-      <c r="P1" s="210" t="s">
+      <c r="P1" s="208" t="s">
         <v>1000</v>
       </c>
-      <c r="Q1" s="210" t="s">
+      <c r="Q1" s="208" t="s">
         <v>999</v>
       </c>
-      <c r="R1" s="211" t="s">
+      <c r="R1" s="209" t="s">
         <v>998</v>
       </c>
-      <c r="S1" s="210" t="s">
+      <c r="S1" s="208" t="s">
         <v>997</v>
       </c>
-      <c r="T1" s="211" t="s">
+      <c r="T1" s="209" t="s">
         <v>996</v>
       </c>
-      <c r="U1" s="211" t="s">
+      <c r="U1" s="209" t="s">
         <v>995</v>
       </c>
-      <c r="V1" s="209" t="s">
+      <c r="V1" s="207" t="s">
         <v>994</v>
       </c>
-      <c r="W1" s="210" t="s">
+      <c r="W1" s="208" t="s">
         <v>993</v>
       </c>
-      <c r="X1" s="210" t="s">
+      <c r="X1" s="208" t="s">
         <v>992</v>
       </c>
-      <c r="Y1" s="210" t="s">
+      <c r="Y1" s="208" t="s">
         <v>991</v>
       </c>
-      <c r="Z1" s="209" t="s">
+      <c r="Z1" s="207" t="s">
         <v>990</v>
       </c>
-      <c r="AA1" s="209" t="s">
+      <c r="AA1" s="207" t="s">
         <v>989</v>
       </c>
-      <c r="AB1" s="208" t="s">
+      <c r="AB1" s="206" t="s">
         <v>988</v>
       </c>
-      <c r="AC1" s="207" t="s">
+      <c r="AC1" s="205" t="s">
         <v>987</v>
       </c>
     </row>
@@ -6989,11 +6943,11 @@
       </c>
       <c r="W2" s="145"/>
       <c r="X2" s="49"/>
-      <c r="Y2" s="205"/>
-      <c r="Z2" s="203" t="s">
+      <c r="Y2" s="203"/>
+      <c r="Z2" s="210" t="s">
         <v>981</v>
       </c>
-      <c r="AA2" s="202"/>
+      <c r="AA2" s="211"/>
       <c r="AB2" s="81"/>
       <c r="AC2" s="80"/>
     </row>
@@ -7012,7 +6966,7 @@
       </c>
       <c r="E3" s="53"/>
       <c r="F3" s="52"/>
-      <c r="G3" s="204"/>
+      <c r="G3" s="202"/>
       <c r="H3" s="177" t="s">
         <v>148</v>
       </c>
@@ -7059,14 +7013,14 @@
       <c r="W3" s="49"/>
       <c r="X3" s="49"/>
       <c r="Y3" s="49"/>
-      <c r="Z3" s="203" t="s">
+      <c r="Z3" s="210" t="s">
         <v>975</v>
       </c>
-      <c r="AA3" s="202"/>
+      <c r="AA3" s="211"/>
       <c r="AB3" s="81"/>
       <c r="AC3" s="80"/>
     </row>
-    <row r="4" spans="1:29" s="30" customFormat="1" ht="112.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" s="30" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="55" t="s">
         <v>962</v>
       </c>
@@ -7153,7 +7107,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="5" spans="1:29" s="30" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" s="30" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="55" t="s">
         <v>948</v>
       </c>
@@ -7240,7 +7194,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="6" spans="1:29" s="131" customFormat="1" ht="72.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" s="131" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A6" s="180" t="s">
         <v>943</v>
       </c>
@@ -7309,7 +7263,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="7" spans="1:29" s="30" customFormat="1" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" s="30" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="55" t="s">
         <v>934</v>
       </c>
@@ -7392,7 +7346,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="8" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="55" t="s">
         <v>924</v>
       </c>
@@ -7475,7 +7429,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="9" spans="1:29" s="131" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" s="131" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A9" s="180" t="s">
         <v>903</v>
       </c>
@@ -7556,7 +7510,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="10" spans="1:29" s="30" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" s="30" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="55" t="s">
         <v>916</v>
       </c>
@@ -7641,7 +7595,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="11" spans="1:29" s="30" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" s="30" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="55" t="s">
         <v>912</v>
       </c>
@@ -7726,7 +7680,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="12" spans="1:29" s="30" customFormat="1" ht="114" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" s="30" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="55" t="s">
         <v>892</v>
       </c>
@@ -7813,7 +7767,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="13" spans="1:29" s="30" customFormat="1" ht="150.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" s="30" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="55" t="s">
         <v>881</v>
       </c>
@@ -7898,7 +7852,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="14" spans="1:29" s="131" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" s="131" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A14" s="180" t="s">
         <v>875</v>
       </c>
@@ -8010,7 +7964,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="16" spans="1:29" s="30" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" s="30" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="55" t="s">
         <v>860</v>
       </c>
@@ -8095,7 +8049,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="17" spans="1:29" s="30" customFormat="1" ht="108.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" s="30" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="55" t="s">
         <v>850</v>
       </c>
@@ -8180,7 +8134,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="18" spans="1:29" s="196" customFormat="1" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" s="196" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="81" t="s">
         <v>840</v>
       </c>
@@ -8261,7 +8215,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="19" spans="1:29" s="138" customFormat="1" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" s="138" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="55" t="s">
         <v>831</v>
       </c>
@@ -8342,7 +8296,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="20" spans="1:29" s="138" customFormat="1" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" s="138" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A20" s="191" t="s">
         <v>824</v>
       </c>
@@ -8395,7 +8349,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="21" spans="1:29" s="30" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A21" s="191" t="s">
         <v>817</v>
       </c>
@@ -8456,7 +8410,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="22" spans="1:29" s="30" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A22" s="191" t="s">
         <v>809</v>
       </c>
@@ -8513,7 +8467,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="23" spans="1:29" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A23" s="191" t="s">
         <v>804</v>
       </c>
@@ -8570,7 +8524,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="24" spans="1:29" s="30" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A24" s="191" t="s">
         <v>797</v>
       </c>
@@ -8627,7 +8581,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="25" spans="1:29" s="105" customFormat="1" ht="157.5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:29" s="105" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="109" t="s">
         <v>795</v>
       </c>
@@ -8710,7 +8664,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="26" spans="1:29" s="105" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:29" s="105" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A26" s="109" t="s">
         <v>790</v>
       </c>
@@ -8793,7 +8747,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="27" spans="1:29" s="138" customFormat="1" ht="157.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:29" s="138" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="55" t="s">
         <v>781</v>
       </c>
@@ -8876,7 +8830,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="28" spans="1:29" s="105" customFormat="1" ht="141.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:29" s="105" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="109" t="s">
         <v>773</v>
       </c>
@@ -8959,7 +8913,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="29" spans="1:29" s="105" customFormat="1" ht="143.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:29" s="105" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="109" t="s">
         <v>769</v>
       </c>
@@ -9042,7 +8996,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="30" spans="1:29" s="138" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:29" s="138" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="55" t="s">
         <v>761</v>
       </c>
@@ -9125,7 +9079,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="31" spans="1:29" s="105" customFormat="1" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:29" s="105" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="109" t="s">
         <v>749</v>
       </c>
@@ -9281,7 +9235,7 @@
       <c r="AB32" s="89"/>
       <c r="AC32" s="98"/>
     </row>
-    <row r="33" spans="1:29" s="85" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:29" s="85" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A33" s="97" t="s">
         <v>733</v>
       </c>
@@ -9354,7 +9308,7 @@
       <c r="AB33" s="89"/>
       <c r="AC33" s="98"/>
     </row>
-    <row r="34" spans="1:29" s="105" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:29" s="105" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A34" s="109" t="s">
         <v>726</v>
       </c>
@@ -9437,7 +9391,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="35" spans="1:29" s="85" customFormat="1" ht="68.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:29" s="85" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A35" s="97" t="s">
         <v>719</v>
       </c>
@@ -9856,7 +9810,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="40" spans="1:29" s="105" customFormat="1" ht="128.44999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:29" s="105" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="109" t="s">
         <v>686</v>
       </c>
@@ -10103,7 +10057,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="43" spans="1:29" s="105" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:29" s="105" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A43" s="109" t="s">
         <v>666</v>
       </c>
@@ -10186,7 +10140,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="44" spans="1:29" s="105" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:29" s="105" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A44" s="109" t="s">
         <v>661</v>
       </c>
@@ -10271,7 +10225,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="45" spans="1:29" s="30" customFormat="1" ht="112.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:29" s="30" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="55" t="s">
         <v>635</v>
       </c>
@@ -10407,7 +10361,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="47" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A47" s="109" t="s">
         <v>628</v>
       </c>
@@ -10492,7 +10446,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="48" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="109" t="s">
         <v>622</v>
       </c>
@@ -10577,7 +10531,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="49" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A49" s="109" t="s">
         <v>612</v>
       </c>
@@ -10658,7 +10612,7 @@
       <c r="AB49" s="71"/>
       <c r="AC49" s="106"/>
     </row>
-    <row r="50" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="109" t="s">
         <v>606</v>
       </c>
@@ -10739,7 +10693,7 @@
       <c r="AB50" s="71"/>
       <c r="AC50" s="106"/>
     </row>
-    <row r="51" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="109" t="s">
         <v>598</v>
       </c>
@@ -10824,7 +10778,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="52" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="109" t="s">
         <v>589</v>
       </c>
@@ -10909,7 +10863,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="53" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A53" s="68" t="s">
         <v>573</v>
       </c>
@@ -10960,7 +10914,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="54" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A54" s="68" t="s">
         <v>567</v>
       </c>
@@ -11011,7 +10965,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="55" spans="1:29" s="176" customFormat="1" ht="146.25" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:29" s="176" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="78" t="s">
         <v>545</v>
       </c>
@@ -11096,7 +11050,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="56" spans="1:29" s="30" customFormat="1" ht="167.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:29" s="30" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="109" t="s">
         <v>558</v>
       </c>
@@ -11181,7 +11135,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="57" spans="1:29" s="105" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:29" s="105" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="68" t="s">
         <v>539</v>
       </c>
@@ -11429,7 +11383,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="61" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A61" s="78" t="s">
         <v>509</v>
       </c>
@@ -11510,7 +11464,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="62" spans="1:29" s="30" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A62" s="78" t="s">
         <v>501</v>
       </c>
@@ -12076,7 +12030,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="70" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A70" s="78" t="s">
         <v>448</v>
       </c>
@@ -12157,7 +12111,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="71" spans="1:29" s="154" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:29" s="154" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="68" t="s">
         <v>442</v>
       </c>
@@ -12441,7 +12395,7 @@
       <c r="AB76" s="57"/>
       <c r="AC76" s="56"/>
     </row>
-    <row r="77" spans="1:29" s="30" customFormat="1" ht="123.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:29" s="30" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="78" t="s">
         <v>420</v>
       </c>
@@ -12524,7 +12478,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="78" spans="1:29" s="30" customFormat="1" ht="123.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:29" s="30" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="78" t="s">
         <v>413</v>
       </c>
@@ -12662,7 +12616,7 @@
       <c r="AB79" s="87"/>
       <c r="AC79" s="151"/>
     </row>
-    <row r="80" spans="1:29" s="85" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:29" s="85" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A80" s="97" t="s">
         <v>395</v>
       </c>
@@ -12717,7 +12671,7 @@
       <c r="AB80" s="87"/>
       <c r="AC80" s="151"/>
     </row>
-    <row r="81" spans="1:29" s="79" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:29" s="79" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="109" t="s">
         <v>389</v>
       </c>
@@ -12786,7 +12740,7 @@
       <c r="AB81" s="48"/>
       <c r="AC81" s="150"/>
     </row>
-    <row r="82" spans="1:29" s="105" customFormat="1" ht="200.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:29" s="105" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="78" t="s">
         <v>373</v>
       </c>
@@ -12938,7 +12892,7 @@
       <c r="AB83" s="48"/>
       <c r="AC83" s="150"/>
     </row>
-    <row r="84" spans="1:29" s="134" customFormat="1" ht="104.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:29" s="134" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A84" s="146" t="s">
         <v>347</v>
       </c>
@@ -13015,7 +12969,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="85" spans="1:29" s="134" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:29" s="134" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A85" s="148" t="s">
         <v>345</v>
       </c>
@@ -13088,7 +13042,7 @@
       <c r="AB85" s="81"/>
       <c r="AC85" s="69"/>
     </row>
-    <row r="86" spans="1:29" s="30" customFormat="1" ht="63.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:29" s="30" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="146" t="s">
         <v>328</v>
       </c>
@@ -13167,7 +13121,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="87" spans="1:29" s="134" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:29" s="134" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A87" s="55" t="s">
         <v>317</v>
       </c>
@@ -13317,7 +13271,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="89" spans="1:29" s="138" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:29" s="138" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A89" s="55" t="s">
         <v>5</v>
       </c>
@@ -13390,7 +13344,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="90" spans="1:29" s="138" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:29" s="138" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A90" s="55" t="s">
         <v>3</v>
       </c>
@@ -14068,7 +14022,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="102" spans="1:78" s="131" customFormat="1" ht="112.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:78" s="131" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="97" t="s">
         <v>219</v>
       </c>
@@ -14145,7 +14099,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="103" spans="1:78" s="85" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:78" s="85" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A103" s="97" t="s">
         <v>213</v>
       </c>
@@ -14222,7 +14176,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="104" spans="1:78" s="85" customFormat="1" ht="112.5" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:78" s="85" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="97" t="s">
         <v>206</v>
       </c>
@@ -14301,7 +14255,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="105" spans="1:78" s="85" customFormat="1" ht="112.5" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:78" s="85" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="97" t="s">
         <v>198</v>
       </c>
@@ -14380,7 +14334,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="106" spans="1:78" s="85" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:78" s="85" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A106" s="97" t="s">
         <v>192</v>
       </c>
@@ -14459,7 +14413,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="107" spans="1:78" s="79" customFormat="1" ht="146.25" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:78" s="79" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="82" t="s">
         <v>178</v>
       </c>
@@ -14672,7 +14626,7 @@
       <c r="BY108" s="85"/>
       <c r="BZ108" s="85"/>
     </row>
-    <row r="109" spans="1:78" s="79" customFormat="1" ht="157.5" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:78" s="79" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="82" t="s">
         <v>163</v>
       </c>
@@ -14887,7 +14841,7 @@
       <c r="BY110" s="85"/>
       <c r="BZ110" s="85"/>
     </row>
-    <row r="111" spans="1:78" s="79" customFormat="1" ht="90" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:78" s="79" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="82" t="s">
         <v>133</v>
       </c>
@@ -15619,7 +15573,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="120" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A120" s="68" t="s">
         <v>57</v>
       </c>
@@ -15719,7 +15673,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="122" spans="1:29" s="30" customFormat="1" ht="96.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:29" s="30" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="78" t="s">
         <v>38</v>
       </c>
@@ -15839,7 +15793,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="124" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A124" s="55" t="s">
         <v>23</v>
       </c>
@@ -15896,7 +15850,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="125" spans="1:29" s="30" customFormat="1" ht="157.5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:29" s="30" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="41" t="s">
         <v>18</v>
       </c>
@@ -15951,7 +15905,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="126" spans="1:29" s="22" customFormat="1" ht="337.5" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:29" s="22" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="23" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Reverted to commit f6c8d96baeab7eb342acf9a1e9ec3c9e887a07bc
</commit_message>
<xml_diff>
--- a/public/data/contractuels.xlsx
+++ b/public/data/contractuels.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pcazenp5\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF295826-E277-482E-A1AB-DD1D8E217CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45497558-F7C5-4661-A2BA-2F523C460164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F3DF298-D4C5-439C-AF3F-C52F546A0520}"/>
+    <workbookView xWindow="-17235" yWindow="2805" windowWidth="21600" windowHeight="11235" xr2:uid="{0F3DF298-D4C5-439C-AF3F-C52F546A0520}"/>
   </bookViews>
   <sheets>
     <sheet name="contractuels" sheetId="2" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">contractuels!$A$1:$BZ$127</definedName>
     <definedName name="CODESTAT">#REF!</definedName>
@@ -6404,6 +6407,12 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -6427,12 +6436,6 @@
     </xf>
     <xf numFmtId="49" fontId="27" fillId="7" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -6454,6 +6457,51 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Corps"/>
+      <sheetName val="Grades"/>
+      <sheetName val="Statuts vacataires d'enseignem"/>
+      <sheetName val="Statuts vacataires"/>
+      <sheetName val="Statuts hébergés"/>
+      <sheetName val="Stat-emploi-pos. sans poste"/>
+      <sheetName val="Triplets"/>
+      <sheetName val="Positions"/>
+      <sheetName val="Modalités sc"/>
+      <sheetName val="Congés-absences"/>
+      <sheetName val="Emplois"/>
+      <sheetName val="Catégories d'emploi (plafond)"/>
+      <sheetName val="UO ED"/>
+      <sheetName val="Etablissements"/>
+      <sheetName val="Actes-visas-article"/>
+      <sheetName val="Diplômes"/>
+      <sheetName val="Mise à jour des référentiels"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6759,124 +6807,122 @@
   <dimension ref="A1:BZ128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="5.7109375" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="132.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="255.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="53.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="29.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="82.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="149.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="28.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="74.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="31.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="47.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="53.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="42.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="50.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="36.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="28.5703125" style="4" customWidth="1"/>
-    <col min="26" max="26" width="37.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="38.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="57.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="28.5703125" style="3" customWidth="1"/>
+    <col min="19" max="19" width="28.5703125" style="4" customWidth="1"/>
+    <col min="20" max="20" width="36.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="28.5703125" style="5" customWidth="1"/>
+    <col min="22" max="22" width="28.5703125" style="3" customWidth="1"/>
+    <col min="23" max="25" width="28.5703125" style="4" customWidth="1"/>
+    <col min="26" max="26" width="28.5703125" style="3" customWidth="1"/>
+    <col min="27" max="27" width="28.5703125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="33.42578125" style="2" customWidth="1"/>
     <col min="30" max="16384" width="5.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="204" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="207" t="s">
+    <row r="1" spans="1:29" s="206" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="209" t="s">
         <v>1015</v>
       </c>
-      <c r="B1" s="208" t="s">
+      <c r="B1" s="210" t="s">
         <v>1014</v>
       </c>
-      <c r="C1" s="207" t="s">
+      <c r="C1" s="209" t="s">
         <v>1013</v>
       </c>
-      <c r="D1" s="207" t="s">
+      <c r="D1" s="209" t="s">
         <v>1012</v>
       </c>
-      <c r="E1" s="207" t="s">
+      <c r="E1" s="209" t="s">
         <v>1011</v>
       </c>
-      <c r="F1" s="207" t="s">
+      <c r="F1" s="209" t="s">
         <v>1010</v>
       </c>
-      <c r="G1" s="207" t="s">
+      <c r="G1" s="209" t="s">
         <v>1009</v>
       </c>
-      <c r="H1" s="207" t="s">
+      <c r="H1" s="209" t="s">
         <v>1008</v>
       </c>
-      <c r="I1" s="207" t="s">
+      <c r="I1" s="209" t="s">
         <v>1007</v>
       </c>
-      <c r="J1" s="207" t="s">
+      <c r="J1" s="209" t="s">
         <v>1006</v>
       </c>
-      <c r="K1" s="207" t="s">
+      <c r="K1" s="209" t="s">
         <v>1005</v>
       </c>
-      <c r="L1" s="208" t="s">
+      <c r="L1" s="210" t="s">
         <v>1004</v>
       </c>
-      <c r="M1" s="208" t="s">
+      <c r="M1" s="210" t="s">
         <v>1003</v>
       </c>
-      <c r="N1" s="208" t="s">
+      <c r="N1" s="210" t="s">
         <v>1002</v>
       </c>
-      <c r="O1" s="208" t="s">
+      <c r="O1" s="210" t="s">
         <v>1001</v>
       </c>
-      <c r="P1" s="208" t="s">
+      <c r="P1" s="210" t="s">
         <v>1000</v>
       </c>
-      <c r="Q1" s="208" t="s">
+      <c r="Q1" s="210" t="s">
         <v>999</v>
       </c>
-      <c r="R1" s="209" t="s">
+      <c r="R1" s="211" t="s">
         <v>998</v>
       </c>
-      <c r="S1" s="208" t="s">
+      <c r="S1" s="210" t="s">
         <v>997</v>
       </c>
-      <c r="T1" s="209" t="s">
+      <c r="T1" s="211" t="s">
         <v>996</v>
       </c>
-      <c r="U1" s="209" t="s">
+      <c r="U1" s="211" t="s">
         <v>995</v>
       </c>
-      <c r="V1" s="207" t="s">
+      <c r="V1" s="209" t="s">
         <v>994</v>
       </c>
-      <c r="W1" s="208" t="s">
+      <c r="W1" s="210" t="s">
         <v>993</v>
       </c>
-      <c r="X1" s="208" t="s">
+      <c r="X1" s="210" t="s">
         <v>992</v>
       </c>
-      <c r="Y1" s="208" t="s">
+      <c r="Y1" s="210" t="s">
         <v>991</v>
       </c>
-      <c r="Z1" s="207" t="s">
+      <c r="Z1" s="209" t="s">
         <v>990</v>
       </c>
-      <c r="AA1" s="207" t="s">
+      <c r="AA1" s="209" t="s">
         <v>989</v>
       </c>
-      <c r="AB1" s="206" t="s">
+      <c r="AB1" s="208" t="s">
         <v>988</v>
       </c>
-      <c r="AC1" s="205" t="s">
+      <c r="AC1" s="207" t="s">
         <v>987</v>
       </c>
     </row>
@@ -6943,11 +6989,11 @@
       </c>
       <c r="W2" s="145"/>
       <c r="X2" s="49"/>
-      <c r="Y2" s="203"/>
-      <c r="Z2" s="210" t="s">
+      <c r="Y2" s="205"/>
+      <c r="Z2" s="203" t="s">
         <v>981</v>
       </c>
-      <c r="AA2" s="211"/>
+      <c r="AA2" s="202"/>
       <c r="AB2" s="81"/>
       <c r="AC2" s="80"/>
     </row>
@@ -6966,7 +7012,7 @@
       </c>
       <c r="E3" s="53"/>
       <c r="F3" s="52"/>
-      <c r="G3" s="202"/>
+      <c r="G3" s="204"/>
       <c r="H3" s="177" t="s">
         <v>148</v>
       </c>
@@ -7013,14 +7059,14 @@
       <c r="W3" s="49"/>
       <c r="X3" s="49"/>
       <c r="Y3" s="49"/>
-      <c r="Z3" s="210" t="s">
+      <c r="Z3" s="203" t="s">
         <v>975</v>
       </c>
-      <c r="AA3" s="211"/>
+      <c r="AA3" s="202"/>
       <c r="AB3" s="81"/>
       <c r="AC3" s="80"/>
     </row>
-    <row r="4" spans="1:29" s="30" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" s="30" customFormat="1" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A4" s="55" t="s">
         <v>962</v>
       </c>
@@ -7107,7 +7153,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="5" spans="1:29" s="30" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" s="30" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="55" t="s">
         <v>948</v>
       </c>
@@ -7194,7 +7240,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="6" spans="1:29" s="131" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" s="131" customFormat="1" ht="72.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="180" t="s">
         <v>943</v>
       </c>
@@ -7263,7 +7309,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="7" spans="1:29" s="30" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" s="30" customFormat="1" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="55" t="s">
         <v>934</v>
       </c>
@@ -7346,7 +7392,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="8" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A8" s="55" t="s">
         <v>924</v>
       </c>
@@ -7429,7 +7475,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="9" spans="1:29" s="131" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" s="131" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="180" t="s">
         <v>903</v>
       </c>
@@ -7510,7 +7556,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="10" spans="1:29" s="30" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" s="30" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A10" s="55" t="s">
         <v>916</v>
       </c>
@@ -7595,7 +7641,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="11" spans="1:29" s="30" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" s="30" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A11" s="55" t="s">
         <v>912</v>
       </c>
@@ -7680,7 +7726,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="12" spans="1:29" s="30" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" s="30" customFormat="1" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="55" t="s">
         <v>892</v>
       </c>
@@ -7767,7 +7813,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="13" spans="1:29" s="30" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" s="30" customFormat="1" ht="150.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="55" t="s">
         <v>881</v>
       </c>
@@ -7852,7 +7898,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="14" spans="1:29" s="131" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" s="131" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A14" s="180" t="s">
         <v>875</v>
       </c>
@@ -7964,7 +8010,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="16" spans="1:29" s="30" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" s="30" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="55" t="s">
         <v>860</v>
       </c>
@@ -8049,7 +8095,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="17" spans="1:29" s="30" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" s="30" customFormat="1" ht="108.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="55" t="s">
         <v>850</v>
       </c>
@@ -8134,7 +8180,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="18" spans="1:29" s="196" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" s="196" customFormat="1" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A18" s="81" t="s">
         <v>840</v>
       </c>
@@ -8215,7 +8261,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="19" spans="1:29" s="138" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" s="138" customFormat="1" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A19" s="55" t="s">
         <v>831</v>
       </c>
@@ -8296,7 +8342,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="20" spans="1:29" s="138" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" s="138" customFormat="1" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="191" t="s">
         <v>824</v>
       </c>
@@ -8349,7 +8395,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="21" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" s="30" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="191" t="s">
         <v>817</v>
       </c>
@@ -8410,7 +8456,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="22" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" s="30" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="191" t="s">
         <v>809</v>
       </c>
@@ -8467,7 +8513,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="23" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:29" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="191" t="s">
         <v>804</v>
       </c>
@@ -8524,7 +8570,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="24" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:29" s="30" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="191" t="s">
         <v>797</v>
       </c>
@@ -8581,7 +8627,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="25" spans="1:29" s="105" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:29" s="105" customFormat="1" ht="157.5" x14ac:dyDescent="0.2">
       <c r="A25" s="109" t="s">
         <v>795</v>
       </c>
@@ -8664,7 +8710,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="26" spans="1:29" s="105" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:29" s="105" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A26" s="109" t="s">
         <v>790</v>
       </c>
@@ -8747,7 +8793,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="27" spans="1:29" s="138" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:29" s="138" customFormat="1" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A27" s="55" t="s">
         <v>781</v>
       </c>
@@ -8830,7 +8876,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="28" spans="1:29" s="105" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:29" s="105" customFormat="1" ht="141.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="109" t="s">
         <v>773</v>
       </c>
@@ -8913,7 +8959,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="29" spans="1:29" s="105" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:29" s="105" customFormat="1" ht="143.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="109" t="s">
         <v>769</v>
       </c>
@@ -8996,7 +9042,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="30" spans="1:29" s="138" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:29" s="138" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A30" s="55" t="s">
         <v>761</v>
       </c>
@@ -9079,7 +9125,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="31" spans="1:29" s="105" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:29" s="105" customFormat="1" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="109" t="s">
         <v>749</v>
       </c>
@@ -9235,7 +9281,7 @@
       <c r="AB32" s="89"/>
       <c r="AC32" s="98"/>
     </row>
-    <row r="33" spans="1:29" s="85" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:29" s="85" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A33" s="97" t="s">
         <v>733</v>
       </c>
@@ -9308,7 +9354,7 @@
       <c r="AB33" s="89"/>
       <c r="AC33" s="98"/>
     </row>
-    <row r="34" spans="1:29" s="105" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:29" s="105" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
       <c r="A34" s="109" t="s">
         <v>726</v>
       </c>
@@ -9391,7 +9437,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="35" spans="1:29" s="85" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:29" s="85" customFormat="1" ht="68.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="97" t="s">
         <v>719</v>
       </c>
@@ -9810,7 +9856,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="40" spans="1:29" s="105" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:29" s="105" customFormat="1" ht="128.44999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="109" t="s">
         <v>686</v>
       </c>
@@ -10057,7 +10103,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="43" spans="1:29" s="105" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:29" s="105" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
       <c r="A43" s="109" t="s">
         <v>666</v>
       </c>
@@ -10140,7 +10186,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="44" spans="1:29" s="105" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:29" s="105" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
       <c r="A44" s="109" t="s">
         <v>661</v>
       </c>
@@ -10225,7 +10271,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="45" spans="1:29" s="30" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:29" s="30" customFormat="1" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A45" s="55" t="s">
         <v>635</v>
       </c>
@@ -10361,7 +10407,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="47" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A47" s="109" t="s">
         <v>628</v>
       </c>
@@ -10446,7 +10492,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="48" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A48" s="109" t="s">
         <v>622</v>
       </c>
@@ -10531,7 +10577,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="49" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A49" s="109" t="s">
         <v>612</v>
       </c>
@@ -10612,7 +10658,7 @@
       <c r="AB49" s="71"/>
       <c r="AC49" s="106"/>
     </row>
-    <row r="50" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A50" s="109" t="s">
         <v>606</v>
       </c>
@@ -10693,7 +10739,7 @@
       <c r="AB50" s="71"/>
       <c r="AC50" s="106"/>
     </row>
-    <row r="51" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A51" s="109" t="s">
         <v>598</v>
       </c>
@@ -10778,7 +10824,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="52" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A52" s="109" t="s">
         <v>589</v>
       </c>
@@ -10863,7 +10909,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="53" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A53" s="68" t="s">
         <v>573</v>
       </c>
@@ -10914,7 +10960,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="54" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A54" s="68" t="s">
         <v>567</v>
       </c>
@@ -10965,7 +11011,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="55" spans="1:29" s="176" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:29" s="176" customFormat="1" ht="146.25" x14ac:dyDescent="0.25">
       <c r="A55" s="78" t="s">
         <v>545</v>
       </c>
@@ -11050,7 +11096,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="56" spans="1:29" s="30" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:29" s="30" customFormat="1" ht="167.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="109" t="s">
         <v>558</v>
       </c>
@@ -11135,7 +11181,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="57" spans="1:29" s="105" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:29" s="105" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A57" s="68" t="s">
         <v>539</v>
       </c>
@@ -11383,7 +11429,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="61" spans="1:29" s="30" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A61" s="78" t="s">
         <v>509</v>
       </c>
@@ -11464,7 +11510,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="62" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:29" s="30" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="78" t="s">
         <v>501</v>
       </c>
@@ -12030,7 +12076,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="70" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:29" s="30" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A70" s="78" t="s">
         <v>448</v>
       </c>
@@ -12111,7 +12157,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="71" spans="1:29" s="154" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:29" s="154" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A71" s="68" t="s">
         <v>442</v>
       </c>
@@ -12395,7 +12441,7 @@
       <c r="AB76" s="57"/>
       <c r="AC76" s="56"/>
     </row>
-    <row r="77" spans="1:29" s="30" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:29" s="30" customFormat="1" ht="123.75" x14ac:dyDescent="0.25">
       <c r="A77" s="78" t="s">
         <v>420</v>
       </c>
@@ -12478,7 +12524,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="78" spans="1:29" s="30" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:29" s="30" customFormat="1" ht="123.75" x14ac:dyDescent="0.25">
       <c r="A78" s="78" t="s">
         <v>413</v>
       </c>
@@ -12616,7 +12662,7 @@
       <c r="AB79" s="87"/>
       <c r="AC79" s="151"/>
     </row>
-    <row r="80" spans="1:29" s="85" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:29" s="85" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A80" s="97" t="s">
         <v>395</v>
       </c>
@@ -12671,7 +12717,7 @@
       <c r="AB80" s="87"/>
       <c r="AC80" s="151"/>
     </row>
-    <row r="81" spans="1:29" s="79" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:29" s="79" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A81" s="109" t="s">
         <v>389</v>
       </c>
@@ -12740,7 +12786,7 @@
       <c r="AB81" s="48"/>
       <c r="AC81" s="150"/>
     </row>
-    <row r="82" spans="1:29" s="105" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:29" s="105" customFormat="1" ht="200.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="78" t="s">
         <v>373</v>
       </c>
@@ -12892,7 +12938,7 @@
       <c r="AB83" s="48"/>
       <c r="AC83" s="150"/>
     </row>
-    <row r="84" spans="1:29" s="134" customFormat="1" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:29" s="134" customFormat="1" ht="104.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="146" t="s">
         <v>347</v>
       </c>
@@ -12969,7 +13015,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="85" spans="1:29" s="134" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:29" s="134" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="148" t="s">
         <v>345</v>
       </c>
@@ -13042,7 +13088,7 @@
       <c r="AB85" s="81"/>
       <c r="AC85" s="69"/>
     </row>
-    <row r="86" spans="1:29" s="30" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:29" s="30" customFormat="1" ht="63.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="146" t="s">
         <v>328</v>
       </c>
@@ -13121,7 +13167,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="87" spans="1:29" s="134" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:29" s="134" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="55" t="s">
         <v>317</v>
       </c>
@@ -13271,7 +13317,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="89" spans="1:29" s="138" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:29" s="138" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A89" s="55" t="s">
         <v>5</v>
       </c>
@@ -13344,7 +13390,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="90" spans="1:29" s="138" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:29" s="138" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A90" s="55" t="s">
         <v>3</v>
       </c>
@@ -14022,7 +14068,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="102" spans="1:78" s="131" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:78" s="131" customFormat="1" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A102" s="97" t="s">
         <v>219</v>
       </c>
@@ -14099,7 +14145,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="103" spans="1:78" s="85" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:78" s="85" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
       <c r="A103" s="97" t="s">
         <v>213</v>
       </c>
@@ -14176,7 +14222,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="104" spans="1:78" s="85" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:78" s="85" customFormat="1" ht="112.5" x14ac:dyDescent="0.2">
       <c r="A104" s="97" t="s">
         <v>206</v>
       </c>
@@ -14255,7 +14301,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="105" spans="1:78" s="85" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:78" s="85" customFormat="1" ht="112.5" x14ac:dyDescent="0.2">
       <c r="A105" s="97" t="s">
         <v>198</v>
       </c>
@@ -14334,7 +14380,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="106" spans="1:78" s="85" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:78" s="85" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
       <c r="A106" s="97" t="s">
         <v>192</v>
       </c>
@@ -14413,7 +14459,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="107" spans="1:78" s="79" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:78" s="79" customFormat="1" ht="146.25" x14ac:dyDescent="0.2">
       <c r="A107" s="82" t="s">
         <v>178</v>
       </c>
@@ -14626,7 +14672,7 @@
       <c r="BY108" s="85"/>
       <c r="BZ108" s="85"/>
     </row>
-    <row r="109" spans="1:78" s="79" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:78" s="79" customFormat="1" ht="157.5" x14ac:dyDescent="0.2">
       <c r="A109" s="82" t="s">
         <v>163</v>
       </c>
@@ -14841,7 +14887,7 @@
       <c r="BY110" s="85"/>
       <c r="BZ110" s="85"/>
     </row>
-    <row r="111" spans="1:78" s="79" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:78" s="79" customFormat="1" ht="90" x14ac:dyDescent="0.2">
       <c r="A111" s="82" t="s">
         <v>133</v>
       </c>
@@ -15573,7 +15619,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="120" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:29" s="30" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A120" s="68" t="s">
         <v>57</v>
       </c>
@@ -15673,7 +15719,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="122" spans="1:29" s="30" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:29" s="30" customFormat="1" ht="96.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="78" t="s">
         <v>38</v>
       </c>
@@ -15793,7 +15839,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="124" spans="1:29" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:29" s="30" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A124" s="55" t="s">
         <v>23</v>
       </c>
@@ -15850,7 +15896,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="125" spans="1:29" s="30" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:29" s="30" customFormat="1" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A125" s="41" t="s">
         <v>18</v>
       </c>
@@ -15905,7 +15951,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="126" spans="1:29" s="22" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:29" s="22" customFormat="1" ht="337.5" x14ac:dyDescent="0.2">
       <c r="A126" s="23" t="s">
         <v>16</v>
       </c>

</xml_diff>